<commit_message>
Update docs; add presentation and test report
Updated several project documents (meeting minutes, progress report, SDD, SPPP, SPPP risk management, and STD) and added two new files: CS673_presentation2_team3.pptx and Manual Testing Report.xlsx. These are binary document changes reflecting content updates and the inclusion of the presentation and manual testing results.
</commit_message>
<xml_diff>
--- a/doc/CS673_SPPP_RiskManagement_team3.xlsx
+++ b/doc/CS673_SPPP_RiskManagement_team3.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="141">
   <si>
     <t>This sheet provides some common risks in student projects. You should check if it applies to your group project. 
 You should also feel free to add other risks. Exemplary analysis is also added.</t>
@@ -81,42 +81,45 @@
     <t>Have not heard from one group member</t>
   </si>
   <si>
+    <t>closed</t>
+  </si>
+  <si>
+    <t>add new team members</t>
+  </si>
+  <si>
+    <t>One or more team members added to group</t>
+  </si>
+  <si>
+    <t>2*2*2= 8</t>
+  </si>
+  <si>
+    <t>Will distribute work load to new member and assign them a leader role.</t>
+  </si>
+  <si>
+    <t>Waiting untill professor has finalized teams.</t>
+  </si>
+  <si>
+    <t>Lack of motivation or responsibility</t>
+  </si>
+  <si>
+    <t>One or more team member is not participating and finish their tasks on time.</t>
+  </si>
+  <si>
+    <t>4*4*4=64</t>
+  </si>
+  <si>
+    <t>Team members who are finishing responsibilities.</t>
+  </si>
+  <si>
+    <t>Weekly meething, check in on progress from everyones responsibility.</t>
+  </si>
+  <si>
+    <t>Keep team members on team timeline and make sure everyone understand their tasks.</t>
+  </si>
+  <si>
     <t>Open</t>
   </si>
   <si>
-    <t>add new team members</t>
-  </si>
-  <si>
-    <t>One or more team members added to group</t>
-  </si>
-  <si>
-    <t>2*2*2= 8</t>
-  </si>
-  <si>
-    <t>Will distribute work load to new member and assign them a leader role.</t>
-  </si>
-  <si>
-    <t>Waiting untill professor has finalized teams.</t>
-  </si>
-  <si>
-    <t>Lack of motivation or responsibility</t>
-  </si>
-  <si>
-    <t>One or more team member is not participating and finish their tasks on time.</t>
-  </si>
-  <si>
-    <t>1*4*4=16</t>
-  </si>
-  <si>
-    <t>Team members who are finishing responsibilities.</t>
-  </si>
-  <si>
-    <t>Weekly meething, check in on progress from everyones responsibility.</t>
-  </si>
-  <si>
-    <t>Keep team members on team timeline and make sure everyone understand their tasks.</t>
-  </si>
-  <si>
     <t>Communication</t>
   </si>
   <si>
@@ -180,6 +183,21 @@
     <t>Consistant code check-in on GitHub.</t>
   </si>
   <si>
+    <t>Merge conflicts in Git branches</t>
+  </si>
+  <si>
+    <t>Multiple developers working on React frontend and backend APIs may create merge conflicts.</t>
+  </si>
+  <si>
+    <t>Configuration Lead</t>
+  </si>
+  <si>
+    <t>Use feature branches, enforce pull request reviews, and merge frequently into development branch.</t>
+  </si>
+  <si>
+    <t>Git branching workflow established in GitHub.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Requirements </t>
   </si>
   <si>
@@ -201,6 +219,21 @@
     <t>constant requirements changes</t>
   </si>
   <si>
+    <t>AI-generated hallucinations</t>
+  </si>
+  <si>
+    <t>AI may generate incorrect or unrealistic test cases not grounded in uploaded product documents.</t>
+  </si>
+  <si>
+    <t>QA Lead and AI integration lead</t>
+  </si>
+  <si>
+    <t>Add retrieval grounding, prompt constraints, and human review before saving generated outputs.</t>
+  </si>
+  <si>
+    <t>Human-in-the-loop review process planned.</t>
+  </si>
+  <si>
     <t>Management</t>
   </si>
   <si>
@@ -213,9 +246,6 @@
     <t>Not enough team meetings to have everyone on the same page.</t>
   </si>
   <si>
-    <t>4*4*4=64</t>
-  </si>
-  <si>
     <t>Team has constant weekly meetings that eveyone can attend.With progress updates.</t>
   </si>
   <si>
@@ -303,6 +333,21 @@
     <t>improper technology stack</t>
   </si>
   <si>
+    <t>Frontend/backend integration mismatch</t>
+  </si>
+  <si>
+    <t>React frontend requests may not match Express backend API responses correctly.</t>
+  </si>
+  <si>
+    <t>Design and implementation leads</t>
+  </si>
+  <si>
+    <t>Define API response formats early and test endpoints continuously during development.</t>
+  </si>
+  <si>
+    <t>API integration testing ongoing</t>
+  </si>
+  <si>
     <t>Messy code</t>
   </si>
   <si>
@@ -324,6 +369,21 @@
     <t>Have feature ready in time for testing. Keep doing functional testing for every feature and don't wait till the end to test.</t>
   </si>
   <si>
+    <t>Insufficient AI output validation</t>
+  </si>
+  <si>
+    <t>AI-generated test cases may appear valid but miss important edge cases or business logic.</t>
+  </si>
+  <si>
+    <t>0613/2026</t>
+  </si>
+  <si>
+    <t>Create manual review workflow and validate outputs against uploaded product requirements</t>
+  </si>
+  <si>
+    <t>QA review process currently being designed.</t>
+  </si>
+  <si>
     <t>Integration and deployment</t>
   </si>
   <si>
@@ -340,6 +400,42 @@
   </si>
   <si>
     <t xml:space="preserve">Weekly meeting to stay on product timeline </t>
+  </si>
+  <si>
+    <t>Schedule</t>
+  </si>
+  <si>
+    <t>AI generation feature not completed before demo</t>
+  </si>
+  <si>
+    <t>AI generation workflow may not be fully stable before the scheduled demo.</t>
+  </si>
+  <si>
+    <t>Entire Team</t>
+  </si>
+  <si>
+    <t>Prioritize minimum viable demo functionality and stabilize core workflow before adding optional features.</t>
+  </si>
+  <si>
+    <t>Current focus is AI generation integration.</t>
+  </si>
+  <si>
+    <t>Security</t>
+  </si>
+  <si>
+    <t>Unsafe file upload handling</t>
+  </si>
+  <si>
+    <t>Uploaded files may contain unsupported formats or malicious content.</t>
+  </si>
+  <si>
+    <t>Security Lead</t>
+  </si>
+  <si>
+    <t>Add file validation, upload restrictions, and secure storage handling.</t>
+  </si>
+  <si>
+    <t>File validation rules implemented for PDFs.</t>
   </si>
   <si>
     <t>The team member who is adding the new feature should be the one who determines what is correct for the new functionality that was added.</t>
@@ -356,7 +452,7 @@
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
     <numFmt numFmtId="165" formatCode="m/d"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="9">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -368,6 +464,22 @@
     <font/>
     <font>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11.0"/>
+      <color rgb="FFFF0000"/>
+    </font>
+    <font>
+      <sz val="11.0"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11.0"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11.0"/>
     </font>
     <font>
       <color rgb="FF000000"/>
@@ -397,7 +509,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="31">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -428,23 +540,56 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="right" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    <xf borderId="0" fillId="2" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="right" readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="right" readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="right" vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right" vertical="bottom"/>
@@ -660,7 +805,7 @@
         <v>27</v>
       </c>
       <c r="D5" s="4">
-        <v>1.0</v>
+        <v>4.0</v>
       </c>
       <c r="E5" s="4">
         <v>4.0</v>
@@ -684,7 +829,7 @@
         <v>31</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="M5" s="6"/>
       <c r="N5" s="6"/>
@@ -704,13 +849,13 @@
     </row>
     <row r="6">
       <c r="A6" s="3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D6" s="4">
         <v>1.0</v>
@@ -722,22 +867,22 @@
         <v>4.0</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I6" s="5">
         <v>46158.0</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="L6" s="3" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="M6" s="6"/>
       <c r="N6" s="6"/>
@@ -758,10 +903,10 @@
     <row r="7">
       <c r="A7" s="9"/>
       <c r="B7" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D7" s="4">
         <v>3.0</v>
@@ -773,7 +918,7 @@
         <v>4.0</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H7" s="3" t="s">
         <v>17</v>
@@ -782,13 +927,13 @@
         <v>46158.0</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="M7" s="6"/>
       <c r="N7" s="6"/>
@@ -809,10 +954,10 @@
     <row r="8">
       <c r="A8" s="3"/>
       <c r="B8" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D8" s="4">
         <v>3.0</v>
@@ -824,22 +969,22 @@
         <v>4.0</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I8" s="5">
         <v>46158.0</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="M8" s="6"/>
       <c r="N8" s="6"/>
@@ -860,10 +1005,10 @@
     <row r="9">
       <c r="A9" s="3"/>
       <c r="B9" s="8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D9" s="4">
         <v>3.0</v>
@@ -875,7 +1020,7 @@
         <v>4.0</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H9" s="3" t="s">
         <v>17</v>
@@ -884,13 +1029,13 @@
         <v>46158.0</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="M9" s="6"/>
       <c r="N9" s="6"/>
@@ -909,41 +1054,39 @@
       <c r="AA9" s="6"/>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="B10" s="2" t="s">
+      <c r="A10" s="3"/>
+      <c r="B10" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="D10" s="4">
+      <c r="D10" s="12">
         <v>3.0</v>
       </c>
-      <c r="E10" s="4">
-        <v>4.0</v>
-      </c>
-      <c r="F10" s="4">
-        <v>4.0</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="I10" s="5">
-        <v>46158.0</v>
-      </c>
-      <c r="J10" s="3" t="s">
+      <c r="E10" s="12">
+        <v>4.0</v>
+      </c>
+      <c r="F10" s="12">
+        <v>4.0</v>
+      </c>
+      <c r="G10" s="12">
+        <v>48.0</v>
+      </c>
+      <c r="H10" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="K10" s="3" t="s">
+      <c r="I10" s="14">
+        <v>46186.0</v>
+      </c>
+      <c r="J10" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="L10" s="3" t="s">
-        <v>20</v>
+      <c r="K10" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="L10" s="13" t="s">
+        <v>32</v>
       </c>
       <c r="M10" s="6"/>
       <c r="N10" s="6"/>
@@ -962,20 +1105,42 @@
       <c r="AA10" s="6"/>
     </row>
     <row r="11">
-      <c r="A11" s="7"/>
+      <c r="A11" s="3" t="s">
+        <v>59</v>
+      </c>
       <c r="B11" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C11" s="7"/>
-      <c r="D11" s="10"/>
-      <c r="E11" s="11"/>
-      <c r="F11" s="11"/>
-      <c r="G11" s="11"/>
-      <c r="H11" s="7"/>
-      <c r="I11" s="5"/>
-      <c r="J11" s="7"/>
-      <c r="K11" s="7"/>
-      <c r="L11" s="3"/>
+        <v>60</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="D11" s="4">
+        <v>3.0</v>
+      </c>
+      <c r="E11" s="4">
+        <v>4.0</v>
+      </c>
+      <c r="F11" s="4">
+        <v>4.0</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I11" s="5">
+        <v>46158.0</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="K11" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="L11" s="3" t="s">
+        <v>32</v>
+      </c>
       <c r="M11" s="6"/>
       <c r="N11" s="6"/>
       <c r="O11" s="6"/>
@@ -995,18 +1160,20 @@
     <row r="12">
       <c r="A12" s="7"/>
       <c r="B12" s="2" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="C12" s="7"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="11"/>
-      <c r="F12" s="11"/>
-      <c r="G12" s="11"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="16"/>
+      <c r="F12" s="16"/>
+      <c r="G12" s="16"/>
       <c r="H12" s="7"/>
       <c r="I12" s="5"/>
       <c r="J12" s="7"/>
       <c r="K12" s="7"/>
-      <c r="L12" s="3"/>
+      <c r="L12" s="3" t="s">
+        <v>20</v>
+      </c>
       <c r="M12" s="6"/>
       <c r="N12" s="6"/>
       <c r="O12" s="6"/>
@@ -1024,17 +1191,15 @@
       <c r="AA12" s="6"/>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="s">
-        <v>60</v>
-      </c>
+      <c r="A13" s="7"/>
       <c r="B13" s="2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="C13" s="7"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="11"/>
-      <c r="G13" s="11"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="16"/>
+      <c r="F13" s="16"/>
+      <c r="G13" s="16"/>
       <c r="H13" s="7"/>
       <c r="I13" s="5"/>
       <c r="J13" s="7"/>
@@ -1058,38 +1223,38 @@
     </row>
     <row r="14">
       <c r="A14" s="7"/>
-      <c r="B14" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="D14" s="4">
-        <v>4.0</v>
-      </c>
-      <c r="E14" s="4">
-        <v>4.0</v>
-      </c>
-      <c r="F14" s="4">
-        <v>4.0</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="H14" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I14" s="5">
-        <v>46158.0</v>
-      </c>
-      <c r="J14" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="K14" s="3" t="s">
+      <c r="B14" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="L14" s="3" t="s">
-        <v>20</v>
+      <c r="C14" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="D14" s="12">
+        <v>4.0</v>
+      </c>
+      <c r="E14" s="12">
+        <v>4.0</v>
+      </c>
+      <c r="F14" s="12">
+        <v>4.0</v>
+      </c>
+      <c r="G14" s="12">
+        <v>64.0</v>
+      </c>
+      <c r="H14" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="I14" s="14">
+        <v>46186.0</v>
+      </c>
+      <c r="J14" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="K14" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="L14" s="13" t="s">
+        <v>32</v>
       </c>
       <c r="M14" s="6"/>
       <c r="N14" s="6"/>
@@ -1108,22 +1273,22 @@
       <c r="AA14" s="6"/>
     </row>
     <row r="15">
-      <c r="A15" s="7"/>
-      <c r="B15" s="8" t="s">
-        <v>67</v>
+      <c r="A15" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>72</v>
       </c>
       <c r="C15" s="7"/>
-      <c r="D15" s="10"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="11"/>
-      <c r="G15" s="11"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="16"/>
+      <c r="F15" s="16"/>
+      <c r="G15" s="16"/>
       <c r="H15" s="7"/>
       <c r="I15" s="5"/>
       <c r="J15" s="7"/>
       <c r="K15" s="7"/>
-      <c r="L15" s="3" t="s">
-        <v>20</v>
-      </c>
+      <c r="L15" s="3"/>
       <c r="M15" s="6"/>
       <c r="N15" s="6"/>
       <c r="O15" s="6"/>
@@ -1141,14 +1306,12 @@
       <c r="AA15" s="6"/>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="s">
-        <v>68</v>
-      </c>
+      <c r="A16" s="7"/>
       <c r="B16" s="2" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="D16" s="4">
         <v>4.0</v>
@@ -1160,20 +1323,22 @@
         <v>4.0</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="H16" s="7"/>
+        <v>28</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="I16" s="5">
         <v>46158.0</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="K16" s="3" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="L16" s="3" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="M16" s="6"/>
       <c r="N16" s="6"/>
@@ -1193,38 +1358,20 @@
     </row>
     <row r="17">
       <c r="A17" s="7"/>
-      <c r="B17" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="D17" s="4">
-        <v>4.0</v>
-      </c>
-      <c r="E17" s="4">
-        <v>4.0</v>
-      </c>
-      <c r="F17" s="4">
-        <v>4.0</v>
-      </c>
-      <c r="G17" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="H17" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="I17" s="5">
-        <v>46158.0</v>
-      </c>
-      <c r="J17" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="K17" s="3" t="s">
+      <c r="B17" s="8" t="s">
         <v>77</v>
       </c>
+      <c r="C17" s="7"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="16"/>
+      <c r="F17" s="16"/>
+      <c r="G17" s="16"/>
+      <c r="H17" s="7"/>
+      <c r="I17" s="5"/>
+      <c r="J17" s="7"/>
+      <c r="K17" s="7"/>
       <c r="L17" s="3" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="M17" s="6"/>
       <c r="N17" s="6"/>
@@ -1243,20 +1390,40 @@
       <c r="AA17" s="6"/>
     </row>
     <row r="18">
-      <c r="A18" s="7"/>
+      <c r="A18" s="3" t="s">
+        <v>78</v>
+      </c>
       <c r="B18" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="C18" s="7"/>
-      <c r="D18" s="10"/>
-      <c r="E18" s="11"/>
-      <c r="F18" s="11"/>
-      <c r="G18" s="11"/>
+        <v>79</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="D18" s="4">
+        <v>4.0</v>
+      </c>
+      <c r="E18" s="4">
+        <v>4.0</v>
+      </c>
+      <c r="F18" s="4">
+        <v>4.0</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>28</v>
+      </c>
       <c r="H18" s="7"/>
-      <c r="I18" s="5"/>
-      <c r="J18" s="7"/>
-      <c r="K18" s="7"/>
-      <c r="L18" s="3"/>
+      <c r="I18" s="5">
+        <v>46158.0</v>
+      </c>
+      <c r="J18" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="K18" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="L18" s="3" t="s">
+        <v>20</v>
+      </c>
       <c r="M18" s="6"/>
       <c r="N18" s="6"/>
       <c r="O18" s="6"/>
@@ -1276,34 +1443,34 @@
     <row r="19">
       <c r="A19" s="7"/>
       <c r="B19" s="2" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="D19" s="4">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="E19" s="4">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="F19" s="4">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>81</v>
+        <v>28</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="I19" s="5">
         <v>46158.0</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="L19" s="3" t="s">
         <v>20</v>
@@ -1327,14 +1494,14 @@
     <row r="20">
       <c r="A20" s="7"/>
       <c r="B20" s="2" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C20" s="7"/>
-      <c r="D20" s="10"/>
-      <c r="E20" s="11"/>
-      <c r="F20" s="11"/>
-      <c r="G20" s="11"/>
-      <c r="H20" s="3"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="16"/>
+      <c r="F20" s="16"/>
+      <c r="G20" s="16"/>
+      <c r="H20" s="7"/>
       <c r="I20" s="5"/>
       <c r="J20" s="7"/>
       <c r="K20" s="7"/>
@@ -1356,38 +1523,36 @@
       <c r="AA20" s="6"/>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="s">
-        <v>86</v>
-      </c>
+      <c r="A21" s="7"/>
       <c r="B21" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D21" s="4">
-        <v>4.0</v>
+        <v>3.0</v>
       </c>
       <c r="E21" s="4">
-        <v>5.0</v>
+        <v>3.0</v>
       </c>
       <c r="F21" s="4">
-        <v>5.0</v>
+        <v>2.0</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="I21" s="5">
         <v>46158.0</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="L21" s="3" t="s">
         <v>20</v>
@@ -1409,20 +1574,22 @@
       <c r="AA21" s="6"/>
     </row>
     <row r="22">
-      <c r="A22" s="3"/>
+      <c r="A22" s="7"/>
       <c r="B22" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C22" s="7"/>
-      <c r="D22" s="10"/>
-      <c r="E22" s="11"/>
-      <c r="F22" s="11"/>
-      <c r="G22" s="11"/>
-      <c r="H22" s="7"/>
+      <c r="D22" s="15"/>
+      <c r="E22" s="16"/>
+      <c r="F22" s="16"/>
+      <c r="G22" s="16"/>
+      <c r="H22" s="3"/>
       <c r="I22" s="5"/>
       <c r="J22" s="7"/>
       <c r="K22" s="7"/>
-      <c r="L22" s="3"/>
+      <c r="L22" s="3" t="s">
+        <v>20</v>
+      </c>
       <c r="M22" s="6"/>
       <c r="N22" s="6"/>
       <c r="O22" s="6"/>
@@ -1440,20 +1607,42 @@
       <c r="AA22" s="6"/>
     </row>
     <row r="23">
-      <c r="A23" s="3"/>
+      <c r="A23" s="3" t="s">
+        <v>96</v>
+      </c>
       <c r="B23" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="C23" s="7"/>
-      <c r="D23" s="10"/>
-      <c r="E23" s="11"/>
-      <c r="F23" s="11"/>
-      <c r="G23" s="11"/>
-      <c r="H23" s="7"/>
-      <c r="I23" s="5"/>
-      <c r="J23" s="7"/>
-      <c r="K23" s="7"/>
-      <c r="L23" s="3"/>
+        <v>97</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="D23" s="4">
+        <v>4.0</v>
+      </c>
+      <c r="E23" s="4">
+        <v>5.0</v>
+      </c>
+      <c r="F23" s="4">
+        <v>5.0</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="H23" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="I23" s="5">
+        <v>46158.0</v>
+      </c>
+      <c r="J23" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="K23" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="L23" s="3" t="s">
+        <v>32</v>
+      </c>
       <c r="M23" s="6"/>
       <c r="N23" s="6"/>
       <c r="O23" s="6"/>
@@ -1471,42 +1660,20 @@
       <c r="AA23" s="6"/>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="s">
-        <v>95</v>
-      </c>
+      <c r="A24" s="3"/>
       <c r="B24" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="C24" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="D24" s="4">
-        <v>4.0</v>
-      </c>
-      <c r="E24" s="4">
-        <v>5.0</v>
-      </c>
-      <c r="F24" s="4">
-        <v>5.0</v>
-      </c>
-      <c r="G24" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="H24" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="I24" s="5">
-        <v>46158.0</v>
-      </c>
-      <c r="J24" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="K24" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="L24" s="3" t="s">
-        <v>20</v>
-      </c>
+        <v>103</v>
+      </c>
+      <c r="C24" s="7"/>
+      <c r="D24" s="15"/>
+      <c r="E24" s="16"/>
+      <c r="F24" s="16"/>
+      <c r="G24" s="16"/>
+      <c r="H24" s="7"/>
+      <c r="I24" s="5"/>
+      <c r="J24" s="7"/>
+      <c r="K24" s="7"/>
+      <c r="L24" s="3"/>
       <c r="M24" s="6"/>
       <c r="N24" s="6"/>
       <c r="O24" s="6"/>
@@ -1524,38 +1691,36 @@
       <c r="AA24" s="6"/>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="B25" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="D25" s="4">
-        <v>4.0</v>
-      </c>
-      <c r="E25" s="4">
-        <v>4.0</v>
-      </c>
-      <c r="F25" s="4">
-        <v>4.0</v>
-      </c>
-      <c r="G25" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="H25" s="3" t="s">
+      <c r="A25" s="3"/>
+      <c r="B25" s="17" t="s">
         <v>104</v>
       </c>
-      <c r="I25" s="5">
-        <v>46158.0</v>
-      </c>
-      <c r="J25" s="3" t="s">
+      <c r="C25" s="11" t="s">
         <v>105</v>
       </c>
-      <c r="K25" s="3" t="s">
+      <c r="D25" s="12">
+        <v>4.0</v>
+      </c>
+      <c r="E25" s="12">
+        <v>4.0</v>
+      </c>
+      <c r="F25" s="12">
+        <v>4.0</v>
+      </c>
+      <c r="G25" s="12">
+        <v>64.0</v>
+      </c>
+      <c r="H25" s="13" t="s">
         <v>106</v>
+      </c>
+      <c r="I25" s="14">
+        <v>46186.0</v>
+      </c>
+      <c r="J25" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="K25" s="13" t="s">
+        <v>108</v>
       </c>
       <c r="L25" s="3" t="s">
         <v>20</v>
@@ -1577,18 +1742,20 @@
       <c r="AA25" s="6"/>
     </row>
     <row r="26">
-      <c r="A26" s="2"/>
-      <c r="B26" s="9"/>
+      <c r="A26" s="3"/>
+      <c r="B26" s="2" t="s">
+        <v>109</v>
+      </c>
       <c r="C26" s="7"/>
-      <c r="D26" s="10"/>
-      <c r="E26" s="11"/>
-      <c r="F26" s="11"/>
-      <c r="G26" s="11"/>
+      <c r="D26" s="15"/>
+      <c r="E26" s="16"/>
+      <c r="F26" s="16"/>
+      <c r="G26" s="16"/>
       <c r="H26" s="7"/>
-      <c r="I26" s="13"/>
+      <c r="I26" s="5"/>
       <c r="J26" s="7"/>
       <c r="K26" s="7"/>
-      <c r="L26" s="7"/>
+      <c r="L26" s="3"/>
       <c r="M26" s="6"/>
       <c r="N26" s="6"/>
       <c r="O26" s="6"/>
@@ -1606,17 +1773,42 @@
       <c r="AA26" s="6"/>
     </row>
     <row r="27">
-      <c r="A27" s="14"/>
-      <c r="C27" s="6"/>
-      <c r="D27" s="15"/>
-      <c r="E27" s="16"/>
-      <c r="F27" s="16"/>
-      <c r="G27" s="16"/>
-      <c r="H27" s="6"/>
-      <c r="I27" s="17"/>
-      <c r="J27" s="18"/>
-      <c r="K27" s="6"/>
-      <c r="L27" s="6"/>
+      <c r="A27" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="B27" s="18" t="s">
+        <v>111</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="D27" s="4">
+        <v>4.0</v>
+      </c>
+      <c r="E27" s="4">
+        <v>5.0</v>
+      </c>
+      <c r="F27" s="4">
+        <v>5.0</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="H27" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="I27" s="5">
+        <v>46158.0</v>
+      </c>
+      <c r="J27" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="K27" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="L27" s="3" t="s">
+        <v>32</v>
+      </c>
       <c r="M27" s="6"/>
       <c r="N27" s="6"/>
       <c r="O27" s="6"/>
@@ -1634,17 +1826,40 @@
       <c r="AA27" s="6"/>
     </row>
     <row r="28">
-      <c r="A28" s="14"/>
-      <c r="C28" s="6"/>
-      <c r="D28" s="16"/>
-      <c r="E28" s="16"/>
-      <c r="F28" s="16"/>
-      <c r="G28" s="16"/>
-      <c r="H28" s="6"/>
-      <c r="I28" s="17"/>
-      <c r="J28" s="6"/>
-      <c r="K28" s="6"/>
-      <c r="L28" s="6"/>
+      <c r="A28" s="3"/>
+      <c r="B28" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="C28" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="D28" s="12">
+        <v>5.0</v>
+      </c>
+      <c r="E28" s="12">
+        <v>5.0</v>
+      </c>
+      <c r="F28" s="12">
+        <v>5.0</v>
+      </c>
+      <c r="G28" s="12">
+        <v>125.0</v>
+      </c>
+      <c r="H28" s="13" t="s">
+        <v>113</v>
+      </c>
+      <c r="I28" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="J28" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="K28" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="L28" s="13" t="s">
+        <v>32</v>
+      </c>
       <c r="M28" s="6"/>
       <c r="N28" s="6"/>
       <c r="O28" s="6"/>
@@ -1662,17 +1877,42 @@
       <c r="AA28" s="6"/>
     </row>
     <row r="29">
-      <c r="A29" s="6"/>
-      <c r="C29" s="6"/>
-      <c r="D29" s="16"/>
-      <c r="E29" s="16"/>
-      <c r="F29" s="16"/>
-      <c r="G29" s="16"/>
-      <c r="H29" s="6"/>
-      <c r="I29" s="17"/>
-      <c r="J29" s="18"/>
-      <c r="K29" s="6"/>
-      <c r="L29" s="6"/>
+      <c r="A29" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="B29" s="19" t="s">
+        <v>122</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="D29" s="4">
+        <v>4.0</v>
+      </c>
+      <c r="E29" s="4">
+        <v>4.0</v>
+      </c>
+      <c r="F29" s="4">
+        <v>4.0</v>
+      </c>
+      <c r="G29" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="H29" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="I29" s="5">
+        <v>46158.0</v>
+      </c>
+      <c r="J29" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="K29" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="L29" s="3" t="s">
+        <v>32</v>
+      </c>
       <c r="M29" s="6"/>
       <c r="N29" s="6"/>
       <c r="O29" s="6"/>
@@ -1690,17 +1930,42 @@
       <c r="AA29" s="6"/>
     </row>
     <row r="30">
-      <c r="A30" s="6"/>
-      <c r="C30" s="6"/>
-      <c r="D30" s="16"/>
-      <c r="E30" s="16"/>
-      <c r="F30" s="16"/>
-      <c r="G30" s="16"/>
-      <c r="H30" s="6"/>
-      <c r="I30" s="17"/>
-      <c r="J30" s="18"/>
-      <c r="K30" s="19"/>
-      <c r="L30" s="19"/>
+      <c r="A30" s="17" t="s">
+        <v>127</v>
+      </c>
+      <c r="B30" s="17" t="s">
+        <v>128</v>
+      </c>
+      <c r="C30" s="20" t="s">
+        <v>129</v>
+      </c>
+      <c r="D30" s="12">
+        <v>5.0</v>
+      </c>
+      <c r="E30" s="12">
+        <v>5.0</v>
+      </c>
+      <c r="F30" s="12">
+        <v>4.0</v>
+      </c>
+      <c r="G30" s="12">
+        <v>100.0</v>
+      </c>
+      <c r="H30" s="13" t="s">
+        <v>130</v>
+      </c>
+      <c r="I30" s="21">
+        <v>46186.0</v>
+      </c>
+      <c r="J30" s="13" t="s">
+        <v>131</v>
+      </c>
+      <c r="K30" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="L30" s="13" t="s">
+        <v>32</v>
+      </c>
       <c r="M30" s="6"/>
       <c r="N30" s="6"/>
       <c r="O30" s="6"/>
@@ -1718,17 +1983,42 @@
       <c r="AA30" s="6"/>
     </row>
     <row r="31">
-      <c r="A31" s="6"/>
-      <c r="C31" s="6"/>
-      <c r="D31" s="16"/>
-      <c r="E31" s="16"/>
-      <c r="F31" s="16"/>
-      <c r="G31" s="16"/>
-      <c r="H31" s="6"/>
-      <c r="I31" s="17"/>
-      <c r="J31" s="18"/>
-      <c r="K31" s="6"/>
-      <c r="L31" s="6"/>
+      <c r="A31" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="B31" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="C31" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="D31" s="22">
+        <v>4.0</v>
+      </c>
+      <c r="E31" s="22">
+        <v>5.0</v>
+      </c>
+      <c r="F31" s="22">
+        <v>4.0</v>
+      </c>
+      <c r="G31" s="22">
+        <v>80.0</v>
+      </c>
+      <c r="H31" s="23" t="s">
+        <v>136</v>
+      </c>
+      <c r="I31" s="24">
+        <v>46186.0</v>
+      </c>
+      <c r="J31" s="25" t="s">
+        <v>137</v>
+      </c>
+      <c r="K31" s="23" t="s">
+        <v>138</v>
+      </c>
+      <c r="L31" s="23" t="s">
+        <v>32</v>
+      </c>
       <c r="M31" s="6"/>
       <c r="N31" s="6"/>
       <c r="O31" s="6"/>
@@ -1746,17 +2036,17 @@
       <c r="AA31" s="6"/>
     </row>
     <row r="32">
-      <c r="A32" s="6"/>
+      <c r="A32" s="26"/>
       <c r="C32" s="6"/>
-      <c r="D32" s="16"/>
-      <c r="E32" s="16"/>
-      <c r="F32" s="16"/>
-      <c r="G32" s="16"/>
+      <c r="D32" s="27"/>
+      <c r="E32" s="27"/>
+      <c r="F32" s="27"/>
+      <c r="G32" s="27"/>
       <c r="H32" s="6"/>
-      <c r="I32" s="17"/>
-      <c r="J32" s="18"/>
-      <c r="K32" s="19"/>
-      <c r="L32" s="19"/>
+      <c r="I32" s="28"/>
+      <c r="J32" s="6"/>
+      <c r="K32" s="6"/>
+      <c r="L32" s="6"/>
       <c r="M32" s="6"/>
       <c r="N32" s="6"/>
       <c r="O32" s="6"/>
@@ -1776,16 +2066,16 @@
     <row r="33">
       <c r="A33" s="6"/>
       <c r="C33" s="6"/>
-      <c r="D33" s="16"/>
-      <c r="E33" s="16"/>
-      <c r="F33" s="16"/>
-      <c r="G33" s="16"/>
+      <c r="D33" s="27"/>
+      <c r="E33" s="27"/>
+      <c r="F33" s="27"/>
+      <c r="G33" s="27"/>
       <c r="H33" s="6"/>
-      <c r="I33" s="17"/>
-      <c r="J33" s="18"/>
-      <c r="K33" s="19"/>
-      <c r="L33" s="19"/>
-      <c r="M33" s="19"/>
+      <c r="I33" s="28"/>
+      <c r="J33" s="29"/>
+      <c r="K33" s="6"/>
+      <c r="L33" s="6"/>
+      <c r="M33" s="6"/>
       <c r="N33" s="6"/>
       <c r="O33" s="6"/>
       <c r="P33" s="6"/>
@@ -1803,17 +2093,16 @@
     </row>
     <row r="34">
       <c r="A34" s="6"/>
-      <c r="B34" s="6"/>
       <c r="C34" s="6"/>
-      <c r="D34" s="6"/>
-      <c r="E34" s="6"/>
-      <c r="F34" s="6"/>
-      <c r="G34" s="6"/>
+      <c r="D34" s="27"/>
+      <c r="E34" s="27"/>
+      <c r="F34" s="27"/>
+      <c r="G34" s="27"/>
       <c r="H34" s="6"/>
-      <c r="I34" s="6"/>
-      <c r="J34" s="6"/>
-      <c r="K34" s="6"/>
-      <c r="L34" s="6"/>
+      <c r="I34" s="28"/>
+      <c r="J34" s="29"/>
+      <c r="K34" s="30"/>
+      <c r="L34" s="30"/>
       <c r="M34" s="6"/>
       <c r="N34" s="6"/>
       <c r="O34" s="6"/>
@@ -1831,16 +2120,15 @@
       <c r="AA34" s="6"/>
     </row>
     <row r="35">
-      <c r="A35" s="7"/>
-      <c r="B35" s="7"/>
-      <c r="C35" s="7"/>
-      <c r="D35" s="16"/>
-      <c r="E35" s="16"/>
-      <c r="F35" s="16"/>
-      <c r="G35" s="6"/>
+      <c r="A35" s="6"/>
+      <c r="C35" s="6"/>
+      <c r="D35" s="27"/>
+      <c r="E35" s="27"/>
+      <c r="F35" s="27"/>
+      <c r="G35" s="27"/>
       <c r="H35" s="6"/>
-      <c r="I35" s="6"/>
-      <c r="J35" s="7"/>
+      <c r="I35" s="28"/>
+      <c r="J35" s="29"/>
       <c r="K35" s="6"/>
       <c r="L35" s="6"/>
       <c r="M35" s="6"/>
@@ -1860,18 +2148,17 @@
       <c r="AA35" s="6"/>
     </row>
     <row r="36">
-      <c r="A36" s="7"/>
-      <c r="B36" s="7"/>
-      <c r="C36" s="7"/>
-      <c r="D36" s="16"/>
-      <c r="E36" s="16"/>
-      <c r="F36" s="16"/>
-      <c r="G36" s="6"/>
+      <c r="A36" s="6"/>
+      <c r="C36" s="6"/>
+      <c r="D36" s="27"/>
+      <c r="E36" s="27"/>
+      <c r="F36" s="27"/>
+      <c r="G36" s="27"/>
       <c r="H36" s="6"/>
-      <c r="I36" s="6"/>
-      <c r="J36" s="7"/>
-      <c r="K36" s="6"/>
-      <c r="L36" s="6"/>
+      <c r="I36" s="28"/>
+      <c r="J36" s="29"/>
+      <c r="K36" s="30"/>
+      <c r="L36" s="30"/>
       <c r="M36" s="6"/>
       <c r="N36" s="6"/>
       <c r="O36" s="6"/>
@@ -1889,19 +2176,18 @@
       <c r="AA36" s="6"/>
     </row>
     <row r="37">
-      <c r="A37" s="7"/>
-      <c r="B37" s="7"/>
-      <c r="C37" s="7"/>
-      <c r="D37" s="16"/>
-      <c r="E37" s="16"/>
-      <c r="F37" s="16"/>
-      <c r="G37" s="6"/>
+      <c r="A37" s="6"/>
+      <c r="C37" s="6"/>
+      <c r="D37" s="27"/>
+      <c r="E37" s="27"/>
+      <c r="F37" s="27"/>
+      <c r="G37" s="27"/>
       <c r="H37" s="6"/>
-      <c r="I37" s="6"/>
-      <c r="J37" s="7"/>
-      <c r="K37" s="6"/>
-      <c r="L37" s="6"/>
-      <c r="M37" s="6"/>
+      <c r="I37" s="28"/>
+      <c r="J37" s="29"/>
+      <c r="K37" s="30"/>
+      <c r="L37" s="30"/>
+      <c r="M37" s="30"/>
       <c r="N37" s="6"/>
       <c r="O37" s="6"/>
       <c r="P37" s="6"/>
@@ -1918,16 +2204,16 @@
       <c r="AA37" s="6"/>
     </row>
     <row r="38">
-      <c r="A38" s="7"/>
-      <c r="B38" s="7"/>
-      <c r="C38" s="7"/>
-      <c r="D38" s="16"/>
-      <c r="E38" s="16"/>
-      <c r="F38" s="16"/>
+      <c r="A38" s="6"/>
+      <c r="B38" s="6"/>
+      <c r="C38" s="6"/>
+      <c r="D38" s="6"/>
+      <c r="E38" s="6"/>
+      <c r="F38" s="6"/>
       <c r="G38" s="6"/>
       <c r="H38" s="6"/>
       <c r="I38" s="6"/>
-      <c r="J38" s="7"/>
+      <c r="J38" s="6"/>
       <c r="K38" s="6"/>
       <c r="L38" s="6"/>
       <c r="M38" s="6"/>
@@ -1948,15 +2234,15 @@
     </row>
     <row r="39">
       <c r="A39" s="7"/>
-      <c r="D39" s="16"/>
-      <c r="E39" s="16"/>
-      <c r="F39" s="16"/>
+      <c r="B39" s="7"/>
+      <c r="C39" s="7"/>
+      <c r="D39" s="27"/>
+      <c r="E39" s="27"/>
+      <c r="F39" s="27"/>
       <c r="G39" s="6"/>
       <c r="H39" s="6"/>
       <c r="I39" s="6"/>
-      <c r="J39" s="7" t="s">
-        <v>107</v>
-      </c>
+      <c r="J39" s="7"/>
       <c r="K39" s="6"/>
       <c r="L39" s="6"/>
       <c r="M39" s="6"/>
@@ -1979,15 +2265,13 @@
       <c r="A40" s="7"/>
       <c r="B40" s="7"/>
       <c r="C40" s="7"/>
-      <c r="D40" s="16"/>
-      <c r="E40" s="16"/>
-      <c r="F40" s="16"/>
+      <c r="D40" s="27"/>
+      <c r="E40" s="27"/>
+      <c r="F40" s="27"/>
       <c r="G40" s="6"/>
       <c r="H40" s="6"/>
       <c r="I40" s="6"/>
-      <c r="J40" s="7" t="s">
-        <v>108</v>
-      </c>
+      <c r="J40" s="7"/>
       <c r="K40" s="6"/>
       <c r="L40" s="6"/>
       <c r="M40" s="6"/>
@@ -2010,9 +2294,9 @@
       <c r="A41" s="7"/>
       <c r="B41" s="7"/>
       <c r="C41" s="7"/>
-      <c r="D41" s="16"/>
-      <c r="E41" s="6"/>
-      <c r="F41" s="6"/>
+      <c r="D41" s="27"/>
+      <c r="E41" s="27"/>
+      <c r="F41" s="27"/>
       <c r="G41" s="6"/>
       <c r="H41" s="6"/>
       <c r="I41" s="6"/>
@@ -2036,16 +2320,16 @@
       <c r="AA41" s="6"/>
     </row>
     <row r="42">
-      <c r="A42" s="6"/>
-      <c r="B42" s="6"/>
-      <c r="C42" s="6"/>
-      <c r="D42" s="6"/>
-      <c r="E42" s="6"/>
-      <c r="F42" s="6"/>
+      <c r="A42" s="7"/>
+      <c r="B42" s="7"/>
+      <c r="C42" s="7"/>
+      <c r="D42" s="27"/>
+      <c r="E42" s="27"/>
+      <c r="F42" s="27"/>
       <c r="G42" s="6"/>
       <c r="H42" s="6"/>
       <c r="I42" s="6"/>
-      <c r="J42" s="6"/>
+      <c r="J42" s="7"/>
       <c r="K42" s="6"/>
       <c r="L42" s="6"/>
       <c r="M42" s="6"/>
@@ -2064,20 +2348,51 @@
       <c r="Z42" s="6"/>
       <c r="AA42" s="6"/>
     </row>
+    <row r="43">
+      <c r="A43" s="7"/>
+      <c r="D43" s="27"/>
+      <c r="E43" s="27"/>
+      <c r="F43" s="27"/>
+      <c r="G43" s="6"/>
+      <c r="H43" s="6"/>
+      <c r="I43" s="6"/>
+      <c r="J43" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="K43" s="6"/>
+      <c r="L43" s="6"/>
+      <c r="M43" s="6"/>
+      <c r="N43" s="6"/>
+      <c r="O43" s="6"/>
+      <c r="P43" s="6"/>
+      <c r="Q43" s="6"/>
+      <c r="R43" s="6"/>
+      <c r="S43" s="6"/>
+      <c r="T43" s="6"/>
+      <c r="U43" s="6"/>
+      <c r="V43" s="6"/>
+      <c r="W43" s="6"/>
+      <c r="X43" s="6"/>
+      <c r="Y43" s="6"/>
+      <c r="Z43" s="6"/>
+      <c r="AA43" s="6"/>
+    </row>
     <row r="44">
-      <c r="A44" s="6"/>
-      <c r="B44" s="6"/>
+      <c r="A44" s="7"/>
+      <c r="B44" s="7"/>
       <c r="C44" s="7"/>
-      <c r="D44" s="16"/>
-      <c r="E44" s="16"/>
-      <c r="F44" s="6"/>
-      <c r="G44" s="16"/>
+      <c r="D44" s="27"/>
+      <c r="E44" s="27"/>
+      <c r="F44" s="27"/>
+      <c r="G44" s="6"/>
       <c r="H44" s="6"/>
       <c r="I44" s="6"/>
-      <c r="J44" s="18"/>
-      <c r="K44" s="19"/>
-      <c r="L44" s="19"/>
-      <c r="M44" s="19"/>
+      <c r="J44" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="K44" s="6"/>
+      <c r="L44" s="6"/>
+      <c r="M44" s="6"/>
       <c r="N44" s="6"/>
       <c r="O44" s="6"/>
       <c r="P44" s="6"/>
@@ -2094,17 +2409,17 @@
       <c r="AA44" s="6"/>
     </row>
     <row r="45">
-      <c r="A45" s="6"/>
-      <c r="B45" s="6"/>
+      <c r="A45" s="7"/>
+      <c r="B45" s="7"/>
       <c r="C45" s="7"/>
-      <c r="D45" s="16"/>
-      <c r="E45" s="16"/>
+      <c r="D45" s="27"/>
+      <c r="E45" s="6"/>
       <c r="F45" s="6"/>
-      <c r="G45" s="16"/>
+      <c r="G45" s="6"/>
       <c r="H45" s="6"/>
       <c r="I45" s="6"/>
-      <c r="J45" s="18"/>
-      <c r="K45" s="19"/>
+      <c r="J45" s="7"/>
+      <c r="K45" s="6"/>
       <c r="L45" s="6"/>
       <c r="M45" s="6"/>
       <c r="N45" s="6"/>
@@ -2125,11 +2440,11 @@
     <row r="46">
       <c r="A46" s="6"/>
       <c r="B46" s="6"/>
-      <c r="C46" s="7"/>
-      <c r="D46" s="16"/>
-      <c r="E46" s="16"/>
+      <c r="C46" s="6"/>
+      <c r="D46" s="6"/>
+      <c r="E46" s="6"/>
       <c r="F46" s="6"/>
-      <c r="G46" s="16"/>
+      <c r="G46" s="6"/>
       <c r="H46" s="6"/>
       <c r="I46" s="6"/>
       <c r="J46" s="6"/>
@@ -2151,34 +2466,121 @@
       <c r="Z46" s="6"/>
       <c r="AA46" s="6"/>
     </row>
-    <row r="47">
-      <c r="A47" s="6"/>
-      <c r="B47" s="6"/>
-      <c r="C47" s="7"/>
-      <c r="D47" s="16"/>
-      <c r="E47" s="16"/>
-      <c r="F47" s="6"/>
-      <c r="G47" s="16"/>
-      <c r="H47" s="6"/>
-      <c r="I47" s="6"/>
-      <c r="J47" s="6"/>
-      <c r="K47" s="6"/>
-      <c r="L47" s="6"/>
-      <c r="M47" s="6"/>
-      <c r="N47" s="6"/>
-      <c r="O47" s="6"/>
-      <c r="P47" s="6"/>
-      <c r="Q47" s="6"/>
-      <c r="R47" s="6"/>
-      <c r="S47" s="6"/>
-      <c r="T47" s="6"/>
-      <c r="U47" s="6"/>
-      <c r="V47" s="6"/>
-      <c r="W47" s="6"/>
-      <c r="X47" s="6"/>
-      <c r="Y47" s="6"/>
-      <c r="Z47" s="6"/>
-      <c r="AA47" s="6"/>
+    <row r="48">
+      <c r="A48" s="6"/>
+      <c r="B48" s="6"/>
+      <c r="C48" s="7"/>
+      <c r="D48" s="27"/>
+      <c r="E48" s="27"/>
+      <c r="F48" s="6"/>
+      <c r="G48" s="27"/>
+      <c r="H48" s="6"/>
+      <c r="I48" s="6"/>
+      <c r="J48" s="29"/>
+      <c r="K48" s="30"/>
+      <c r="L48" s="30"/>
+      <c r="M48" s="30"/>
+      <c r="N48" s="6"/>
+      <c r="O48" s="6"/>
+      <c r="P48" s="6"/>
+      <c r="Q48" s="6"/>
+      <c r="R48" s="6"/>
+      <c r="S48" s="6"/>
+      <c r="T48" s="6"/>
+      <c r="U48" s="6"/>
+      <c r="V48" s="6"/>
+      <c r="W48" s="6"/>
+      <c r="X48" s="6"/>
+      <c r="Y48" s="6"/>
+      <c r="Z48" s="6"/>
+      <c r="AA48" s="6"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="6"/>
+      <c r="B49" s="6"/>
+      <c r="C49" s="7"/>
+      <c r="D49" s="27"/>
+      <c r="E49" s="27"/>
+      <c r="F49" s="6"/>
+      <c r="G49" s="27"/>
+      <c r="H49" s="6"/>
+      <c r="I49" s="6"/>
+      <c r="J49" s="29"/>
+      <c r="K49" s="30"/>
+      <c r="L49" s="6"/>
+      <c r="M49" s="6"/>
+      <c r="N49" s="6"/>
+      <c r="O49" s="6"/>
+      <c r="P49" s="6"/>
+      <c r="Q49" s="6"/>
+      <c r="R49" s="6"/>
+      <c r="S49" s="6"/>
+      <c r="T49" s="6"/>
+      <c r="U49" s="6"/>
+      <c r="V49" s="6"/>
+      <c r="W49" s="6"/>
+      <c r="X49" s="6"/>
+      <c r="Y49" s="6"/>
+      <c r="Z49" s="6"/>
+      <c r="AA49" s="6"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="6"/>
+      <c r="B50" s="6"/>
+      <c r="C50" s="7"/>
+      <c r="D50" s="27"/>
+      <c r="E50" s="27"/>
+      <c r="F50" s="6"/>
+      <c r="G50" s="27"/>
+      <c r="H50" s="6"/>
+      <c r="I50" s="6"/>
+      <c r="J50" s="6"/>
+      <c r="K50" s="6"/>
+      <c r="L50" s="6"/>
+      <c r="M50" s="6"/>
+      <c r="N50" s="6"/>
+      <c r="O50" s="6"/>
+      <c r="P50" s="6"/>
+      <c r="Q50" s="6"/>
+      <c r="R50" s="6"/>
+      <c r="S50" s="6"/>
+      <c r="T50" s="6"/>
+      <c r="U50" s="6"/>
+      <c r="V50" s="6"/>
+      <c r="W50" s="6"/>
+      <c r="X50" s="6"/>
+      <c r="Y50" s="6"/>
+      <c r="Z50" s="6"/>
+      <c r="AA50" s="6"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="6"/>
+      <c r="B51" s="6"/>
+      <c r="C51" s="7"/>
+      <c r="D51" s="27"/>
+      <c r="E51" s="27"/>
+      <c r="F51" s="6"/>
+      <c r="G51" s="27"/>
+      <c r="H51" s="6"/>
+      <c r="I51" s="6"/>
+      <c r="J51" s="6"/>
+      <c r="K51" s="6"/>
+      <c r="L51" s="6"/>
+      <c r="M51" s="6"/>
+      <c r="N51" s="6"/>
+      <c r="O51" s="6"/>
+      <c r="P51" s="6"/>
+      <c r="Q51" s="6"/>
+      <c r="R51" s="6"/>
+      <c r="S51" s="6"/>
+      <c r="T51" s="6"/>
+      <c r="U51" s="6"/>
+      <c r="V51" s="6"/>
+      <c r="W51" s="6"/>
+      <c r="X51" s="6"/>
+      <c r="Y51" s="6"/>
+      <c r="Z51" s="6"/>
+      <c r="AA51" s="6"/>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>

</xml_diff>